<commit_message>
People & Work audit: owner decisions carry the R11 defaults (hours, proof, repeat failure, drafts, server report)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T49gnSNZq31rPRt1vHk4Rc
</commit_message>
<xml_diff>
--- a/nexidoc/Nexi_People_Work_Audit_v22.28.xlsx
+++ b/nexidoc/Nexi_People_Work_Audit_v22.28.xlsx
@@ -25,7 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Syra'!$A$1:$M$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Screens'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Engine issues'!$A$1:$H$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Owner decisions'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Owner decisions'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -10655,13 +10655,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10682,6 +10683,11 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t>Until answered</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
@@ -10694,7 +10700,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Edelyn’s and Joshane’s role files are marked DRAFT. Confirm every duty, deadline and proof (or send the corrected files).</t>
+          <t>Edelyn’s and Joshane’s role files are marked DRAFT (Joshane’s has no source file; Edelyn’s comes from JD Rev 0). Confirm every duty, deadline and proof, or send the corrected files.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -10703,6 +10709,11 @@
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Today their duties are generated, scored and listed in the 17:45 report. Proposed until confirmed: keep generating them but leave them out of the score and the report.</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -10726,6 +10737,11 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>Deadline unchanged.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
@@ -10738,7 +10754,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Saturday is off for all five. Should any duty run on a Saturday (e.g. logistics), and should Philippine regular / special holidays skip duties (S29)?</t>
+          <t>Working days for duties: Saturday off and Sunday on for all five. Should Philippine regular / special holidays skip duties (11 duties fall on a holiday Oct–Dec 2026)?</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -10747,6 +10763,11 @@
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Saturday off, Sunday on; an approved per-person work schedule wins; holidays skip duties once S29 ships.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -10760,7 +10781,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Scoring: D = 1, L (late the same day) = 0.5, X = 0; G ≥ 95 %, A ≥ 85 %, R below. Confirm, or give the new weights.</t>
+          <t>Hours: Rea’s start 07:00 or 07:30? Mea’s D01 opening walk-through 06:45 (role file) or 07:15 (Nexi)? Syra’s working hours?</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -10769,6 +10790,11 @@
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Deadlines unchanged until answered.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -10782,15 +10808,20 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Proof types per duty (photo, file, signed sheet, Nexi record) for the U-code (S05) — who accepts proof: the reviewer named in the role file?</t>
+          <t>Scoring: today D = 1, L (late the same day) = 0.5, X = 0; green ≥ 95 %, amber 85–94 %, red below. Confirm, or give new weights.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Eyal</t>
+          <t>Eyal / Dr Amy</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -10804,7 +10835,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Server-sent 17:45 fail report (S63) and server-side per-user task filtering (S64) need a Cloudflare deploy — approve when ready.</t>
+          <t>Proof: what counts as proof per duty (S05)?</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10814,12 +10845,71 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
+          <t>A file or an SOS / QuickBooks / case reference; a note alone = U (unverified), except Mea D05 and D13 where a note is enough; NA needs a manager.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>OD-07</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Repeat failure: when is a duty a repeat failure (S05)?</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Eyal / Jinky</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Daily: 3 misses in 7 days. Weekly / monthly: 2 in a row.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>OD-08</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Server-sent 17:45 fail report when no manager has Nexi open (S63): who receives it and who acknowledges it by 09:00? Server-side per-user task filtering (S64)?</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Eyal</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Not deployed until Eyal says yes (both need a Cloudflare deploy).</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D7"/>
+  <autoFilter ref="A1:E9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>